<commit_message>
Phase 1: Bleu's first pass on terms and style, exported to TSV
tools/export-decisions.ps1 reads the yellow columns of work/terminology-decisions.xlsx into work/decisions-terms.tsv and work/decisions-style.tsv, so decisions can be diffed and read by the other tools.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/terminology-decisions.xlsx
+++ b/work/terminology-decisions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maost\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\[01] Martin\[07] Claude Code\NS2-Spanish-Translation\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23CAC15F-CF6F-40D2-93E2-ED219A262548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F525CB-A8B7-43D0-B805-3BD385715403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5220" yWindow="0" windowWidth="14070" windowHeight="13845" xr2:uid="{6146A626-7569-4F77-96CD-9013D1E3384E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{6146A626-7569-4F77-96CD-9013D1E3384E}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="746">
   <si>
     <t>Category</t>
   </si>
@@ -2090,6 +2090,198 @@
   </si>
   <si>
     <t>Style questions left</t>
+  </si>
+  <si>
+    <t>OK as suggested</t>
+  </si>
+  <si>
+    <t>la</t>
+  </si>
+  <si>
+    <t>can't think for now of a context where juego would be distinctively preferable.</t>
+  </si>
+  <si>
+    <t>I don't like Desarrollar in this context. RTS games in spanish tend to use 'investigar'</t>
+  </si>
+  <si>
+    <t>¿No hay usos o 'jurisprudencia' de esto por ejemplo en el tutorial?</t>
+  </si>
+  <si>
+    <t>nodo de res</t>
+  </si>
+  <si>
+    <t>el</t>
+  </si>
+  <si>
+    <t>I saw "Res" used also in the translation so this could work too since res is such a common ns2 term</t>
+  </si>
+  <si>
+    <t>árbol de tecnologías</t>
+  </si>
+  <si>
+    <t>ELO</t>
+  </si>
+  <si>
+    <t>Buscar referencias de que se usa en juegos como CSGO, Dota, etc</t>
+  </si>
+  <si>
+    <t>partida rápida</t>
+  </si>
+  <si>
+    <t>partida competitiva</t>
+  </si>
+  <si>
+    <t>No debería unificarse con command station?</t>
+  </si>
+  <si>
+    <t>granada de racimo</t>
+  </si>
+  <si>
+    <t>granada de pulso</t>
+  </si>
+  <si>
+    <t>nano-escudo</t>
+  </si>
+  <si>
+    <t>Beacon de emergencia</t>
+  </si>
+  <si>
+    <t>armamento avanzado</t>
+  </si>
+  <si>
+    <t>soporte avanzado</t>
+  </si>
+  <si>
+    <t>portal de fase</t>
+  </si>
+  <si>
+    <t>tecnología de fase</t>
+  </si>
+  <si>
+    <t>propulsores</t>
+  </si>
+  <si>
+    <t>los</t>
+  </si>
+  <si>
+    <t>asiento de eyección</t>
+  </si>
+  <si>
+    <t>placas de armadura</t>
+  </si>
+  <si>
+    <t>las</t>
+  </si>
+  <si>
+    <t>campo  de nano-escudo</t>
+  </si>
+  <si>
+    <t>campo de catalyst</t>
+  </si>
+  <si>
+    <t>campo de regen</t>
+  </si>
+  <si>
+    <t>el juego base usa chamber?</t>
+  </si>
+  <si>
+    <t>chamber de evolución</t>
+  </si>
+  <si>
+    <t>contaminación</t>
+  </si>
+  <si>
+    <t>biomasa</t>
+  </si>
+  <si>
+    <t>morder</t>
+  </si>
+  <si>
+    <t>parásito</t>
+  </si>
+  <si>
+    <t>ver contexto?</t>
+  </si>
+  <si>
+    <t>escupitajo</t>
+  </si>
+  <si>
+    <t>depende de si es verbo o sustantivo</t>
+  </si>
+  <si>
+    <t>spray de curación</t>
+  </si>
+  <si>
+    <t>espinas</t>
+  </si>
+  <si>
+    <t>esporas</t>
+  </si>
+  <si>
+    <t>enzima</t>
+  </si>
+  <si>
+    <t>membrana mucosa</t>
+  </si>
+  <si>
+    <t>halucinación</t>
+  </si>
+  <si>
+    <t>bruma de ocultamiento</t>
+  </si>
+  <si>
+    <t>neblina de nutrientes</t>
+  </si>
+  <si>
+    <t>ruptura</t>
+  </si>
+  <si>
+    <t>eco</t>
+  </si>
+  <si>
+    <t>tinta</t>
+  </si>
+  <si>
+    <t>caparazón</t>
+  </si>
+  <si>
+    <t>regeneración</t>
+  </si>
+  <si>
+    <t>vampirismo</t>
+  </si>
+  <si>
+    <t>camuflage</t>
+  </si>
+  <si>
+    <t>foco</t>
+  </si>
+  <si>
+    <t>celeridad</t>
+  </si>
+  <si>
+    <t>adrenalina</t>
+  </si>
+  <si>
+    <t>As suggested</t>
+  </si>
+  <si>
+    <t>presiona</t>
+  </si>
+  <si>
+    <t>investigar</t>
+  </si>
+  <si>
+    <t>click</t>
+  </si>
+  <si>
+    <t>infinitive. Correct for instructions in sentences which should use imperative.</t>
+  </si>
+  <si>
+    <t>check against popular RTS in spanish</t>
+  </si>
+  <si>
+    <t>To be checked on a case by case basis</t>
   </si>
 </sst>
 </file>
@@ -2640,7 +2832,7 @@
       </c>
       <c r="B14" s="11">
         <f>COUNTA(Terms!L2:L153)</f>
-        <v>0</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -2649,7 +2841,7 @@
       </c>
       <c r="B15" s="11">
         <f>ROWS(Terms!L2:L153)-COUNTA(Terms!L2:L153)</f>
-        <v>152</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -2658,7 +2850,7 @@
       </c>
       <c r="B16" s="11">
         <f>COUNTA(Style!E2:E20)</f>
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -2667,7 +2859,7 @@
       </c>
       <c r="B17" s="11">
         <f>ROWS(Style!E2:E20)-COUNTA(Style!E2:E20)</f>
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2682,9 +2874,7 @@
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="3" max="5" width="18.5703125" customWidth="1"/>
     <col min="6" max="6" width="16.7109375" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" customWidth="1"/>
     <col min="8" max="8" width="34.7109375" customWidth="1"/>
@@ -2774,7 +2964,9 @@
       <c r="K2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="7"/>
+      <c r="L2" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
       <c r="O2" s="8"/>
@@ -2809,7 +3001,9 @@
       <c r="K3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="7"/>
+      <c r="L3" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
       <c r="O3" s="8"/>
@@ -2846,7 +3040,9 @@
       <c r="K4" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="7"/>
+      <c r="L4" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
       <c r="O4" s="8"/>
@@ -2883,7 +3079,9 @@
       <c r="K5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="L5" s="7"/>
+      <c r="L5" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
       <c r="O5" s="8"/>
@@ -2914,7 +3112,9 @@
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="6"/>
-      <c r="L6" s="7"/>
+      <c r="L6" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
       <c r="O6" s="8"/>
@@ -2953,7 +3153,9 @@
       <c r="K7" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="L7" s="7"/>
+      <c r="L7" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="8"/>
@@ -2992,7 +3194,9 @@
       <c r="K8" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L8" s="7"/>
+      <c r="L8" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="8"/>
@@ -3029,7 +3233,9 @@
       <c r="K9" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="L9" s="7"/>
+      <c r="L9" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
       <c r="O9" s="8"/>
@@ -3062,7 +3268,9 @@
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="6"/>
-      <c r="L10" s="7"/>
+      <c r="L10" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
       <c r="O10" s="8"/>
@@ -3101,7 +3309,9 @@
       <c r="K11" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="L11" s="7"/>
+      <c r="L11" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>
       <c r="O11" s="8"/>
@@ -3140,12 +3350,14 @@
       <c r="K12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="L12" s="7"/>
+      <c r="L12" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
       <c r="O12" s="8"/>
     </row>
-    <row r="13" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -3179,10 +3391,18 @@
       <c r="K13" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="8"/>
+      <c r="L13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="O13" s="8" t="s">
+        <v>684</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
@@ -3216,7 +3436,9 @@
       <c r="K14" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="L14" s="7"/>
+      <c r="L14" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
       <c r="O14" s="8"/>
@@ -3253,7 +3475,9 @@
       <c r="K15" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="L15" s="7"/>
+      <c r="L15" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
       <c r="O15" s="8"/>
@@ -3290,7 +3514,9 @@
       <c r="K16" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="L16" s="7"/>
+      <c r="L16" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
       <c r="O16" s="8"/>
@@ -3327,7 +3553,9 @@
       <c r="K17" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="L17" s="7"/>
+      <c r="L17" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
       <c r="O17" s="8"/>
@@ -3358,7 +3586,9 @@
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="6"/>
-      <c r="L18" s="7"/>
+      <c r="L18" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
       <c r="O18" s="8"/>
@@ -3395,7 +3625,9 @@
       <c r="K19" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="L19" s="7"/>
+      <c r="L19" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
       <c r="O19" s="8"/>
@@ -3430,7 +3662,9 @@
       <c r="K20" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="L20" s="7"/>
+      <c r="L20" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
       <c r="O20" s="8"/>
@@ -3467,7 +3701,9 @@
       <c r="K21" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="L21" s="7"/>
+      <c r="L21" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M21" s="7"/>
       <c r="N21" s="7"/>
       <c r="O21" s="8"/>
@@ -3506,7 +3742,9 @@
       <c r="K22" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="L22" s="7"/>
+      <c r="L22" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
       <c r="O22" s="8"/>
@@ -3545,12 +3783,14 @@
       <c r="K23" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="L23" s="7"/>
+      <c r="L23" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M23" s="7"/>
       <c r="N23" s="7"/>
       <c r="O23" s="8"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>15</v>
       </c>
@@ -3582,12 +3822,16 @@
       <c r="K24" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="L24" s="7"/>
+      <c r="L24" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M24" s="7"/>
       <c r="N24" s="7"/>
-      <c r="O24" s="8"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O24" s="8" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
@@ -3616,7 +3860,9 @@
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
-      <c r="O25" s="8"/>
+      <c r="O25" s="8" t="s">
+        <v>686</v>
+      </c>
     </row>
     <row r="26" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
@@ -3652,10 +3898,18 @@
       <c r="K26" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="8"/>
+      <c r="L26" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="N26" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="O26" s="8" t="s">
+        <v>689</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
@@ -3683,9 +3937,15 @@
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="6"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7"/>
+      <c r="L27" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="N27" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O27" s="8"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
@@ -3714,12 +3974,14 @@
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="6"/>
-      <c r="L28" s="7"/>
+      <c r="L28" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M28" s="7"/>
       <c r="N28" s="7"/>
       <c r="O28" s="8"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>15</v>
       </c>
@@ -3753,10 +4015,16 @@
       <c r="K29" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="L29" s="7"/>
-      <c r="M29" s="7"/>
+      <c r="L29" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>691</v>
+      </c>
       <c r="N29" s="7"/>
-      <c r="O29" s="8"/>
+      <c r="O29" s="8" t="s">
+        <v>692</v>
+      </c>
     </row>
     <row r="30" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
@@ -3784,9 +4052,15 @@
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="6"/>
-      <c r="L30" s="7"/>
-      <c r="M30" s="7"/>
-      <c r="N30" s="7"/>
+      <c r="L30" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M30" s="7" t="s">
+        <v>693</v>
+      </c>
+      <c r="N30" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O30" s="8"/>
     </row>
     <row r="31" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -3815,9 +4089,15 @@
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="6"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
+      <c r="L31" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M31" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="N31" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O31" s="8"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
@@ -3852,7 +4132,9 @@
       <c r="K32" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="L32" s="7"/>
+      <c r="L32" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M32" s="7"/>
       <c r="N32" s="7"/>
       <c r="O32" s="8"/>
@@ -3889,7 +4171,9 @@
       <c r="K33" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="L33" s="7"/>
+      <c r="L33" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
       <c r="O33" s="8"/>
@@ -3924,7 +4208,9 @@
       <c r="K34" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="L34" s="7"/>
+      <c r="L34" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M34" s="7"/>
       <c r="N34" s="7"/>
       <c r="O34" s="8"/>
@@ -3961,12 +4247,14 @@
       <c r="K35" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="L35" s="7"/>
+      <c r="L35" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M35" s="7"/>
       <c r="N35" s="7"/>
       <c r="O35" s="8"/>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>165</v>
       </c>
@@ -3990,10 +4278,14 @@
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="6"/>
-      <c r="L36" s="7"/>
+      <c r="L36" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
-      <c r="O36" s="8"/>
+      <c r="O36" s="8" t="s">
+        <v>695</v>
+      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
@@ -4025,7 +4317,9 @@
       <c r="K37" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="L37" s="7"/>
+      <c r="L37" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
       <c r="O37" s="8"/>
@@ -4062,7 +4356,9 @@
       <c r="K38" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="L38" s="7"/>
+      <c r="L38" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M38" s="7"/>
       <c r="N38" s="7"/>
       <c r="O38" s="8"/>
@@ -4097,7 +4393,9 @@
       <c r="K39" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="L39" s="7"/>
+      <c r="L39" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
       <c r="O39" s="8"/>
@@ -4132,7 +4430,9 @@
       <c r="K40" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="L40" s="7"/>
+      <c r="L40" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M40" s="7"/>
       <c r="N40" s="7"/>
       <c r="O40" s="8"/>
@@ -4167,7 +4467,9 @@
       <c r="K41" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="L41" s="7"/>
+      <c r="L41" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M41" s="7"/>
       <c r="N41" s="7"/>
       <c r="O41" s="8"/>
@@ -4202,9 +4504,15 @@
       <c r="K42" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="L42" s="7"/>
-      <c r="M42" s="7"/>
-      <c r="N42" s="7"/>
+      <c r="L42" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M42" s="7" t="s">
+        <v>702</v>
+      </c>
+      <c r="N42" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O42" s="8"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.2">
@@ -4231,7 +4539,9 @@
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
       <c r="K43" s="6"/>
-      <c r="L43" s="7"/>
+      <c r="L43" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
       <c r="O43" s="8"/>
@@ -4260,7 +4570,9 @@
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
       <c r="K44" s="6"/>
-      <c r="L44" s="7"/>
+      <c r="L44" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
       <c r="O44" s="8"/>
@@ -4289,7 +4601,9 @@
       <c r="I45" s="4"/>
       <c r="J45" s="4"/>
       <c r="K45" s="6"/>
-      <c r="L45" s="7"/>
+      <c r="L45" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
       <c r="O45" s="8"/>
@@ -4326,7 +4640,9 @@
       <c r="K46" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="L46" s="7"/>
+      <c r="L46" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
       <c r="O46" s="8"/>
@@ -4361,7 +4677,9 @@
       <c r="K47" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="L47" s="7"/>
+      <c r="L47" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
       <c r="O47" s="8"/>
@@ -4396,7 +4714,9 @@
       <c r="K48" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="L48" s="7"/>
+      <c r="L48" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
       <c r="O48" s="8"/>
@@ -4433,7 +4753,9 @@
       <c r="K49" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="L49" s="7"/>
+      <c r="L49" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
       <c r="O49" s="8"/>
@@ -4468,7 +4790,9 @@
       <c r="K50" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="L50" s="7"/>
+      <c r="L50" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M50" s="7"/>
       <c r="N50" s="7"/>
       <c r="O50" s="8"/>
@@ -4503,7 +4827,9 @@
       <c r="K51" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="L51" s="7"/>
+      <c r="L51" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M51" s="7"/>
       <c r="N51" s="7"/>
       <c r="O51" s="8"/>
@@ -4540,7 +4866,9 @@
       <c r="K52" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="L52" s="7"/>
+      <c r="L52" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
       <c r="O52" s="8"/>
@@ -4575,7 +4903,9 @@
       <c r="K53" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="L53" s="7"/>
+      <c r="L53" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
       <c r="O53" s="8"/>
@@ -4612,7 +4942,9 @@
       <c r="K54" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="L54" s="7"/>
+      <c r="L54" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
       <c r="O54" s="8"/>
@@ -4649,7 +4981,9 @@
       <c r="K55" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="L55" s="7"/>
+      <c r="L55" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M55" s="7"/>
       <c r="N55" s="7"/>
       <c r="O55" s="8"/>
@@ -4686,7 +5020,9 @@
       <c r="K56" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="L56" s="7"/>
+      <c r="L56" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M56" s="7"/>
       <c r="N56" s="7"/>
       <c r="O56" s="8"/>
@@ -4723,7 +5059,9 @@
       <c r="K57" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="L57" s="7"/>
+      <c r="L57" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M57" s="7"/>
       <c r="N57" s="7"/>
       <c r="O57" s="8"/>
@@ -4760,7 +5098,9 @@
       <c r="K58" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="L58" s="7"/>
+      <c r="L58" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M58" s="7"/>
       <c r="N58" s="7"/>
       <c r="O58" s="8"/>
@@ -4799,7 +5139,9 @@
       <c r="K59" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="L59" s="7"/>
+      <c r="L59" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M59" s="7"/>
       <c r="N59" s="7"/>
       <c r="O59" s="8"/>
@@ -4838,7 +5180,9 @@
       <c r="K60" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="L60" s="7"/>
+      <c r="L60" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M60" s="7"/>
       <c r="N60" s="7"/>
       <c r="O60" s="8"/>
@@ -4877,7 +5221,9 @@
       <c r="K61" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="L61" s="7"/>
+      <c r="L61" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M61" s="7"/>
       <c r="N61" s="7"/>
       <c r="O61" s="8"/>
@@ -4910,7 +5256,9 @@
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
       <c r="K62" s="6"/>
-      <c r="L62" s="7"/>
+      <c r="L62" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M62" s="7"/>
       <c r="N62" s="7"/>
       <c r="O62" s="8"/>
@@ -4945,7 +5293,9 @@
       <c r="K63" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="L63" s="7"/>
+      <c r="L63" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M63" s="7"/>
       <c r="N63" s="7"/>
       <c r="O63" s="8"/>
@@ -4980,7 +5330,9 @@
       <c r="K64" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="L64" s="7"/>
+      <c r="L64" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M64" s="7"/>
       <c r="N64" s="7"/>
       <c r="O64" s="8"/>
@@ -5019,7 +5371,9 @@
       <c r="K65" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="L65" s="7"/>
+      <c r="L65" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M65" s="7"/>
       <c r="N65" s="7"/>
       <c r="O65" s="8"/>
@@ -5052,7 +5406,9 @@
       <c r="I66" s="4"/>
       <c r="J66" s="4"/>
       <c r="K66" s="6"/>
-      <c r="L66" s="7"/>
+      <c r="L66" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M66" s="7"/>
       <c r="N66" s="7"/>
       <c r="O66" s="8"/>
@@ -5091,7 +5447,9 @@
       <c r="K67" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="L67" s="7"/>
+      <c r="L67" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M67" s="7"/>
       <c r="N67" s="7"/>
       <c r="O67" s="8"/>
@@ -5122,9 +5480,15 @@
       <c r="I68" s="4"/>
       <c r="J68" s="4"/>
       <c r="K68" s="6"/>
-      <c r="L68" s="7"/>
-      <c r="M68" s="7"/>
-      <c r="N68" s="7"/>
+      <c r="L68" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M68" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="N68" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O68" s="8"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.2">
@@ -5153,9 +5517,15 @@
       <c r="I69" s="4"/>
       <c r="J69" s="4"/>
       <c r="K69" s="6"/>
-      <c r="L69" s="7"/>
-      <c r="M69" s="7"/>
-      <c r="N69" s="7"/>
+      <c r="L69" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M69" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="N69" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O69" s="8"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.2">
@@ -5184,9 +5554,15 @@
       <c r="I70" s="4"/>
       <c r="J70" s="4"/>
       <c r="K70" s="6"/>
-      <c r="L70" s="7"/>
-      <c r="M70" s="7"/>
-      <c r="N70" s="7"/>
+      <c r="L70" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M70" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="N70" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O70" s="8"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.2">
@@ -5215,7 +5591,9 @@
       <c r="I71" s="4"/>
       <c r="J71" s="4"/>
       <c r="K71" s="6"/>
-      <c r="L71" s="7"/>
+      <c r="L71" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M71" s="7"/>
       <c r="N71" s="7"/>
       <c r="O71" s="8"/>
@@ -5244,7 +5622,9 @@
       <c r="I72" s="4"/>
       <c r="J72" s="4"/>
       <c r="K72" s="6"/>
-      <c r="L72" s="7"/>
+      <c r="L72" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M72" s="7"/>
       <c r="N72" s="7"/>
       <c r="O72" s="8"/>
@@ -5275,7 +5655,9 @@
       <c r="I73" s="4"/>
       <c r="J73" s="4"/>
       <c r="K73" s="6"/>
-      <c r="L73" s="7"/>
+      <c r="L73" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M73" s="7"/>
       <c r="N73" s="7"/>
       <c r="O73" s="8"/>
@@ -5306,8 +5688,12 @@
       <c r="I74" s="4"/>
       <c r="J74" s="4"/>
       <c r="K74" s="6"/>
-      <c r="L74" s="7"/>
-      <c r="M74" s="7"/>
+      <c r="L74" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M74" s="7" t="s">
+        <v>698</v>
+      </c>
       <c r="N74" s="7"/>
       <c r="O74" s="8"/>
     </row>
@@ -5337,7 +5723,9 @@
       <c r="I75" s="4"/>
       <c r="J75" s="4"/>
       <c r="K75" s="6"/>
-      <c r="L75" s="7"/>
+      <c r="L75" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M75" s="7"/>
       <c r="N75" s="7"/>
       <c r="O75" s="8"/>
@@ -5372,8 +5760,12 @@
       <c r="K76" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="L76" s="7"/>
-      <c r="M76" s="7"/>
+      <c r="L76" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="M76" s="7" t="s">
+        <v>699</v>
+      </c>
       <c r="N76" s="7"/>
       <c r="O76" s="8"/>
     </row>
@@ -5401,7 +5793,9 @@
       <c r="I77" s="4"/>
       <c r="J77" s="4"/>
       <c r="K77" s="6"/>
-      <c r="L77" s="7"/>
+      <c r="L77" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M77" s="7"/>
       <c r="N77" s="7"/>
       <c r="O77" s="8"/>
@@ -5430,8 +5824,12 @@
       <c r="I78" s="4"/>
       <c r="J78" s="4"/>
       <c r="K78" s="6"/>
-      <c r="L78" s="7"/>
-      <c r="M78" s="7"/>
+      <c r="L78" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M78" s="7" t="s">
+        <v>700</v>
+      </c>
       <c r="N78" s="7"/>
       <c r="O78" s="8"/>
     </row>
@@ -5459,8 +5857,12 @@
       <c r="I79" s="4"/>
       <c r="J79" s="4"/>
       <c r="K79" s="6"/>
-      <c r="L79" s="7"/>
-      <c r="M79" s="7"/>
+      <c r="L79" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M79" s="7" t="s">
+        <v>701</v>
+      </c>
       <c r="N79" s="7"/>
       <c r="O79" s="8"/>
     </row>
@@ -5494,8 +5896,12 @@
       <c r="K80" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="L80" s="7"/>
-      <c r="M80" s="7"/>
+      <c r="L80" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M80" s="7" t="s">
+        <v>703</v>
+      </c>
       <c r="N80" s="7"/>
       <c r="O80" s="8"/>
     </row>
@@ -5533,7 +5939,9 @@
       <c r="K81" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="L81" s="7"/>
+      <c r="L81" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M81" s="7"/>
       <c r="N81" s="7"/>
       <c r="O81" s="8"/>
@@ -5572,7 +5980,9 @@
       <c r="K82" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="L82" s="7"/>
+      <c r="L82" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M82" s="7"/>
       <c r="N82" s="7"/>
       <c r="O82" s="8"/>
@@ -5609,9 +6019,15 @@
       <c r="K83" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="L83" s="7"/>
-      <c r="M83" s="7"/>
-      <c r="N83" s="7"/>
+      <c r="L83" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M83" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="N83" s="7" t="s">
+        <v>705</v>
+      </c>
       <c r="O83" s="8"/>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.2">
@@ -5638,9 +6054,15 @@
       <c r="I84" s="4"/>
       <c r="J84" s="4"/>
       <c r="K84" s="6"/>
-      <c r="L84" s="7"/>
-      <c r="M84" s="7"/>
-      <c r="N84" s="7"/>
+      <c r="L84" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M84" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="N84" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O84" s="8"/>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.2">
@@ -5667,9 +6089,15 @@
       <c r="I85" s="4"/>
       <c r="J85" s="4"/>
       <c r="K85" s="6"/>
-      <c r="L85" s="7"/>
-      <c r="M85" s="7"/>
-      <c r="N85" s="7"/>
+      <c r="L85" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M85" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="N85" s="7" t="s">
+        <v>708</v>
+      </c>
       <c r="O85" s="8"/>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.2">
@@ -5696,9 +6124,15 @@
       <c r="I86" s="4"/>
       <c r="J86" s="4"/>
       <c r="K86" s="6"/>
-      <c r="L86" s="7"/>
-      <c r="M86" s="7"/>
-      <c r="N86" s="7"/>
+      <c r="L86" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M86" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="N86" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O86" s="8"/>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.2">
@@ -5725,9 +6159,15 @@
       <c r="I87" s="4"/>
       <c r="J87" s="4"/>
       <c r="K87" s="6"/>
-      <c r="L87" s="7"/>
-      <c r="M87" s="7"/>
-      <c r="N87" s="7"/>
+      <c r="L87" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="M87" s="7" t="s">
+        <v>710</v>
+      </c>
+      <c r="N87" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O87" s="8"/>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.2">
@@ -5754,9 +6194,15 @@
       <c r="I88" s="4"/>
       <c r="J88" s="4"/>
       <c r="K88" s="6"/>
-      <c r="L88" s="7"/>
-      <c r="M88" s="7"/>
-      <c r="N88" s="7"/>
+      <c r="L88" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="M88" s="7" t="s">
+        <v>711</v>
+      </c>
+      <c r="N88" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O88" s="8"/>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.2">
@@ -5789,7 +6235,9 @@
       <c r="K89" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="L89" s="7"/>
+      <c r="L89" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M89" s="7"/>
       <c r="N89" s="7"/>
       <c r="O89" s="8"/>
@@ -5824,7 +6272,9 @@
       <c r="K90" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="L90" s="7"/>
+      <c r="L90" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M90" s="7"/>
       <c r="N90" s="7"/>
       <c r="O90" s="8"/>
@@ -5859,7 +6309,9 @@
       <c r="K91" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="L91" s="7"/>
+      <c r="L91" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M91" s="7"/>
       <c r="N91" s="7"/>
       <c r="O91" s="8"/>
@@ -5894,7 +6346,9 @@
       <c r="K92" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="L92" s="7"/>
+      <c r="L92" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M92" s="7"/>
       <c r="N92" s="7"/>
       <c r="O92" s="8"/>
@@ -5929,7 +6383,9 @@
       <c r="K93" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="L93" s="7"/>
+      <c r="L93" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M93" s="7"/>
       <c r="N93" s="7"/>
       <c r="O93" s="8"/>
@@ -5960,7 +6416,9 @@
       <c r="I94" s="4"/>
       <c r="J94" s="4"/>
       <c r="K94" s="6"/>
-      <c r="L94" s="7"/>
+      <c r="L94" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M94" s="7"/>
       <c r="N94" s="7"/>
       <c r="O94" s="8"/>
@@ -5999,7 +6457,9 @@
       <c r="K95" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="L95" s="7"/>
+      <c r="L95" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M95" s="7"/>
       <c r="N95" s="7"/>
       <c r="O95" s="8"/>
@@ -6034,7 +6494,9 @@
       <c r="K96" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="L96" s="7"/>
+      <c r="L96" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M96" s="7"/>
       <c r="N96" s="7"/>
       <c r="O96" s="8"/>
@@ -6069,7 +6531,9 @@
       <c r="K97" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="L97" s="7"/>
+      <c r="L97" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M97" s="7"/>
       <c r="N97" s="7"/>
       <c r="O97" s="8"/>
@@ -6104,7 +6568,9 @@
       <c r="K98" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="L98" s="7"/>
+      <c r="L98" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M98" s="7"/>
       <c r="N98" s="7"/>
       <c r="O98" s="8"/>
@@ -6139,7 +6605,9 @@
       <c r="K99" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="L99" s="7"/>
+      <c r="L99" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M99" s="7"/>
       <c r="N99" s="7"/>
       <c r="O99" s="8"/>
@@ -6172,7 +6640,9 @@
       <c r="I100" s="4"/>
       <c r="J100" s="4"/>
       <c r="K100" s="6"/>
-      <c r="L100" s="7"/>
+      <c r="L100" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M100" s="7"/>
       <c r="N100" s="7"/>
       <c r="O100" s="8"/>
@@ -6201,7 +6671,9 @@
       <c r="I101" s="4"/>
       <c r="J101" s="4"/>
       <c r="K101" s="6"/>
-      <c r="L101" s="7"/>
+      <c r="L101" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M101" s="7"/>
       <c r="N101" s="7"/>
       <c r="O101" s="8"/>
@@ -6238,7 +6710,9 @@
       <c r="K102" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="L102" s="7"/>
+      <c r="L102" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M102" s="7"/>
       <c r="N102" s="7"/>
       <c r="O102" s="8"/>
@@ -6275,7 +6749,9 @@
       <c r="K103" s="6" t="s">
         <v>410</v>
       </c>
-      <c r="L103" s="7"/>
+      <c r="L103" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M103" s="7"/>
       <c r="N103" s="7"/>
       <c r="O103" s="8"/>
@@ -6312,7 +6788,9 @@
       <c r="K104" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="L104" s="7"/>
+      <c r="L104" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M104" s="7"/>
       <c r="N104" s="7"/>
       <c r="O104" s="8"/>
@@ -6347,7 +6825,9 @@
       <c r="K105" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="L105" s="7"/>
+      <c r="L105" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M105" s="7"/>
       <c r="N105" s="7"/>
       <c r="O105" s="8"/>
@@ -6382,7 +6862,9 @@
       <c r="K106" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="L106" s="7"/>
+      <c r="L106" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M106" s="7"/>
       <c r="N106" s="7"/>
       <c r="O106" s="8"/>
@@ -6417,7 +6899,9 @@
       <c r="K107" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="L107" s="7"/>
+      <c r="L107" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M107" s="7"/>
       <c r="N107" s="7"/>
       <c r="O107" s="8"/>
@@ -6452,7 +6936,9 @@
       <c r="K108" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="L108" s="7"/>
+      <c r="L108" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M108" s="7"/>
       <c r="N108" s="7"/>
       <c r="O108" s="8"/>
@@ -6487,7 +6973,9 @@
       <c r="K109" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="L109" s="7"/>
+      <c r="L109" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M109" s="7"/>
       <c r="N109" s="7"/>
       <c r="O109" s="8"/>
@@ -6522,7 +7010,9 @@
       <c r="K110" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="L110" s="7"/>
+      <c r="L110" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M110" s="7"/>
       <c r="N110" s="7"/>
       <c r="O110" s="8"/>
@@ -6557,7 +7047,9 @@
       <c r="K111" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="L111" s="7"/>
+      <c r="L111" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M111" s="7"/>
       <c r="N111" s="7"/>
       <c r="O111" s="8"/>
@@ -6591,7 +7083,9 @@
       <c r="L112" s="7"/>
       <c r="M112" s="7"/>
       <c r="N112" s="7"/>
-      <c r="O112" s="8"/>
+      <c r="O112" s="8" t="s">
+        <v>712</v>
+      </c>
     </row>
     <row r="113" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="s">
@@ -6627,7 +7121,9 @@
       <c r="K113" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="L113" s="7"/>
+      <c r="L113" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M113" s="7"/>
       <c r="N113" s="7"/>
       <c r="O113" s="8"/>
@@ -6656,9 +7152,15 @@
       <c r="I114" s="4"/>
       <c r="J114" s="4"/>
       <c r="K114" s="6"/>
-      <c r="L114" s="7"/>
-      <c r="M114" s="7"/>
-      <c r="N114" s="7"/>
+      <c r="L114" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="M114" s="7" t="s">
+        <v>713</v>
+      </c>
+      <c r="N114" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O114" s="8"/>
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.2">
@@ -6685,9 +7187,15 @@
       <c r="I115" s="4"/>
       <c r="J115" s="4"/>
       <c r="K115" s="6"/>
-      <c r="L115" s="7"/>
-      <c r="M115" s="7"/>
-      <c r="N115" s="7"/>
+      <c r="L115" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M115" s="7" t="s">
+        <v>714</v>
+      </c>
+      <c r="N115" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O115" s="8"/>
     </row>
     <row r="116" spans="1:15" x14ac:dyDescent="0.2">
@@ -6724,7 +7232,9 @@
       <c r="K116" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="L116" s="7"/>
+      <c r="L116" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M116" s="7"/>
       <c r="N116" s="7"/>
       <c r="O116" s="8"/>
@@ -6761,9 +7271,15 @@
       <c r="K117" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="L117" s="7"/>
-      <c r="M117" s="7"/>
-      <c r="N117" s="7"/>
+      <c r="L117" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M117" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="N117" s="7" t="s">
+        <v>683</v>
+      </c>
       <c r="O117" s="8"/>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.2">
@@ -6798,7 +7314,9 @@
       <c r="K118" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="L118" s="7"/>
+      <c r="L118" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M118" s="7"/>
       <c r="N118" s="7"/>
       <c r="O118" s="8"/>
@@ -6833,10 +7351,16 @@
       <c r="K119" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="L119" s="7"/>
-      <c r="M119" s="7"/>
+      <c r="L119" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M119" s="7" t="s">
+        <v>716</v>
+      </c>
       <c r="N119" s="7"/>
-      <c r="O119" s="8"/>
+      <c r="O119" s="8" t="s">
+        <v>718</v>
+      </c>
     </row>
     <row r="120" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A120" s="3" t="s">
@@ -6868,7 +7392,9 @@
       <c r="K120" s="6" t="s">
         <v>479</v>
       </c>
-      <c r="L120" s="7"/>
+      <c r="L120" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M120" s="7"/>
       <c r="N120" s="7"/>
       <c r="O120" s="8"/>
@@ -6903,9 +7429,15 @@
       <c r="K121" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="L121" s="7"/>
-      <c r="M121" s="7"/>
-      <c r="N121" s="7"/>
+      <c r="L121" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M121" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="N121" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O121" s="8"/>
     </row>
     <row r="122" spans="1:15" ht="51" x14ac:dyDescent="0.2">
@@ -6938,7 +7470,9 @@
       <c r="K122" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="L122" s="7"/>
+      <c r="L122" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M122" s="7"/>
       <c r="N122" s="7"/>
       <c r="O122" s="8"/>
@@ -6973,10 +7507,18 @@
       <c r="K123" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="L123" s="7"/>
-      <c r="M123" s="7"/>
-      <c r="N123" s="7"/>
-      <c r="O123" s="8"/>
+      <c r="L123" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M123" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="N123" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="O123" s="8" t="s">
+        <v>720</v>
+      </c>
     </row>
     <row r="124" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A124" s="3" t="s">
@@ -7008,9 +7550,15 @@
       <c r="K124" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="L124" s="7"/>
-      <c r="M124" s="7"/>
-      <c r="N124" s="7"/>
+      <c r="L124" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="M124" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="N124" s="7" t="s">
+        <v>688</v>
+      </c>
       <c r="O124" s="8"/>
     </row>
     <row r="125" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
@@ -7043,7 +7591,9 @@
       <c r="K125" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="L125" s="7"/>
+      <c r="L125" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M125" s="7"/>
       <c r="N125" s="7"/>
       <c r="O125" s="8"/>
@@ -7078,9 +7628,15 @@
       <c r="K126" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="L126" s="7"/>
-      <c r="M126" s="7"/>
-      <c r="N126" s="7"/>
+      <c r="L126" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M126" s="7" t="s">
+        <v>722</v>
+      </c>
+      <c r="N126" s="7" t="s">
+        <v>708</v>
+      </c>
       <c r="O126" s="8"/>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.2">
@@ -7107,9 +7663,15 @@
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
       <c r="K127" s="6"/>
-      <c r="L127" s="7"/>
-      <c r="M127" s="7"/>
-      <c r="N127" s="7"/>
+      <c r="L127" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M127" s="7" t="s">
+        <v>723</v>
+      </c>
+      <c r="N127" s="7" t="s">
+        <v>708</v>
+      </c>
       <c r="O127" s="8"/>
     </row>
     <row r="128" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -7142,7 +7704,9 @@
       <c r="K128" s="6" t="s">
         <v>508</v>
       </c>
-      <c r="L128" s="7"/>
+      <c r="L128" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M128" s="7"/>
       <c r="N128" s="7"/>
       <c r="O128" s="8"/>
@@ -7171,7 +7735,9 @@
       <c r="I129" s="4"/>
       <c r="J129" s="4"/>
       <c r="K129" s="6"/>
-      <c r="L129" s="7"/>
+      <c r="L129" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M129" s="7"/>
       <c r="N129" s="7"/>
       <c r="O129" s="8"/>
@@ -7206,7 +7772,9 @@
       <c r="K130" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="L130" s="7"/>
+      <c r="L130" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M130" s="7"/>
       <c r="N130" s="7"/>
       <c r="O130" s="8"/>
@@ -7241,7 +7809,9 @@
       <c r="K131" s="6" t="s">
         <v>517</v>
       </c>
-      <c r="L131" s="7"/>
+      <c r="L131" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M131" s="7"/>
       <c r="N131" s="7"/>
       <c r="O131" s="8"/>
@@ -7276,7 +7846,9 @@
       <c r="K132" s="6" t="s">
         <v>521</v>
       </c>
-      <c r="L132" s="7"/>
+      <c r="L132" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M132" s="7"/>
       <c r="N132" s="7"/>
       <c r="O132" s="8"/>
@@ -7311,7 +7883,9 @@
       <c r="K133" s="6" t="s">
         <v>525</v>
       </c>
-      <c r="L133" s="7"/>
+      <c r="L133" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M133" s="7"/>
       <c r="N133" s="7"/>
       <c r="O133" s="8"/>
@@ -7346,12 +7920,14 @@
       <c r="K134" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="L134" s="7"/>
+      <c r="L134" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M134" s="7"/>
       <c r="N134" s="7"/>
       <c r="O134" s="8"/>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A135" s="3" t="s">
         <v>471</v>
       </c>
@@ -7384,7 +7960,9 @@
       <c r="L135" s="7"/>
       <c r="M135" s="7"/>
       <c r="N135" s="7"/>
-      <c r="O135" s="8"/>
+      <c r="O135" s="8" t="s">
+        <v>720</v>
+      </c>
     </row>
     <row r="136" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A136" s="3" t="s">
@@ -7418,7 +7996,9 @@
       <c r="K136" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="L136" s="7"/>
+      <c r="L136" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M136" s="7"/>
       <c r="N136" s="7"/>
       <c r="O136" s="8"/>
@@ -7449,8 +8029,12 @@
       <c r="I137" s="4"/>
       <c r="J137" s="4"/>
       <c r="K137" s="6"/>
-      <c r="L137" s="7"/>
-      <c r="M137" s="7"/>
+      <c r="L137" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M137" s="7" t="s">
+        <v>724</v>
+      </c>
       <c r="N137" s="7"/>
       <c r="O137" s="8"/>
     </row>
@@ -7478,8 +8062,12 @@
       <c r="I138" s="4"/>
       <c r="J138" s="4"/>
       <c r="K138" s="6"/>
-      <c r="L138" s="7"/>
-      <c r="M138" s="7"/>
+      <c r="L138" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M138" s="7" t="s">
+        <v>725</v>
+      </c>
       <c r="N138" s="7"/>
       <c r="O138" s="8"/>
     </row>
@@ -7507,8 +8095,12 @@
       <c r="I139" s="4"/>
       <c r="J139" s="4"/>
       <c r="K139" s="6"/>
-      <c r="L139" s="7"/>
-      <c r="M139" s="7"/>
+      <c r="L139" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M139" s="7" t="s">
+        <v>726</v>
+      </c>
       <c r="N139" s="7"/>
       <c r="O139" s="8"/>
     </row>
@@ -7536,8 +8128,12 @@
       <c r="I140" s="4"/>
       <c r="J140" s="4"/>
       <c r="K140" s="6"/>
-      <c r="L140" s="7"/>
-      <c r="M140" s="7"/>
+      <c r="L140" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M140" s="7" t="s">
+        <v>727</v>
+      </c>
       <c r="N140" s="7"/>
       <c r="O140" s="8"/>
     </row>
@@ -7571,8 +8167,12 @@
       <c r="K141" s="6" t="s">
         <v>547</v>
       </c>
-      <c r="L141" s="7"/>
-      <c r="M141" s="7"/>
+      <c r="L141" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M141" s="7" t="s">
+        <v>728</v>
+      </c>
       <c r="N141" s="7"/>
       <c r="O141" s="8"/>
     </row>
@@ -7600,8 +8200,12 @@
       <c r="I142" s="4"/>
       <c r="J142" s="4"/>
       <c r="K142" s="6"/>
-      <c r="L142" s="7"/>
-      <c r="M142" s="7"/>
+      <c r="L142" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M142" s="7" t="s">
+        <v>729</v>
+      </c>
       <c r="N142" s="7"/>
       <c r="O142" s="8"/>
     </row>
@@ -7635,8 +8239,12 @@
       <c r="K143" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="L143" s="7"/>
-      <c r="M143" s="7"/>
+      <c r="L143" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M143" s="7" t="s">
+        <v>730</v>
+      </c>
       <c r="N143" s="7"/>
       <c r="O143" s="8"/>
     </row>
@@ -7670,8 +8278,12 @@
       <c r="K144" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="L144" s="7"/>
-      <c r="M144" s="7"/>
+      <c r="L144" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M144" s="7" t="s">
+        <v>731</v>
+      </c>
       <c r="N144" s="7"/>
       <c r="O144" s="8"/>
     </row>
@@ -7705,8 +8317,12 @@
       <c r="K145" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="L145" s="7"/>
-      <c r="M145" s="7"/>
+      <c r="L145" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M145" s="7" t="s">
+        <v>732</v>
+      </c>
       <c r="N145" s="7"/>
       <c r="O145" s="8"/>
     </row>
@@ -7740,8 +8356,12 @@
       <c r="K146" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="L146" s="7"/>
-      <c r="M146" s="7"/>
+      <c r="L146" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M146" s="7" t="s">
+        <v>733</v>
+      </c>
       <c r="N146" s="7"/>
       <c r="O146" s="8"/>
     </row>
@@ -7769,8 +8389,12 @@
       <c r="I147" s="4"/>
       <c r="J147" s="4"/>
       <c r="K147" s="6"/>
-      <c r="L147" s="7"/>
-      <c r="M147" s="7"/>
+      <c r="L147" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M147" s="7" t="s">
+        <v>734</v>
+      </c>
       <c r="N147" s="7"/>
       <c r="O147" s="8"/>
     </row>
@@ -7798,8 +8422,12 @@
       <c r="I148" s="4"/>
       <c r="J148" s="4"/>
       <c r="K148" s="6"/>
-      <c r="L148" s="7"/>
-      <c r="M148" s="7"/>
+      <c r="L148" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M148" s="7" t="s">
+        <v>735</v>
+      </c>
       <c r="N148" s="7"/>
       <c r="O148" s="8"/>
     </row>
@@ -7833,7 +8461,9 @@
       <c r="K149" s="6" t="s">
         <v>571</v>
       </c>
-      <c r="L149" s="7"/>
+      <c r="L149" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M149" s="7"/>
       <c r="N149" s="7"/>
       <c r="O149" s="8"/>
@@ -7868,8 +8498,12 @@
       <c r="K150" s="6" t="s">
         <v>575</v>
       </c>
-      <c r="L150" s="7"/>
-      <c r="M150" s="7"/>
+      <c r="L150" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M150" s="7" t="s">
+        <v>736</v>
+      </c>
       <c r="N150" s="7"/>
       <c r="O150" s="8"/>
     </row>
@@ -7903,8 +8537,12 @@
       <c r="K151" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="L151" s="7"/>
-      <c r="M151" s="7"/>
+      <c r="L151" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M151" s="7" t="s">
+        <v>737</v>
+      </c>
       <c r="N151" s="7"/>
       <c r="O151" s="8"/>
     </row>
@@ -7938,8 +8576,12 @@
       <c r="K152" s="6" t="s">
         <v>583</v>
       </c>
-      <c r="L152" s="7"/>
-      <c r="M152" s="7"/>
+      <c r="L152" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M152" s="7" t="s">
+        <v>738</v>
+      </c>
       <c r="N152" s="7"/>
       <c r="O152" s="8"/>
     </row>
@@ -7973,13 +8615,29 @@
       <c r="K153" s="6" t="s">
         <v>586</v>
       </c>
-      <c r="L153" s="7"/>
+      <c r="L153" s="7" t="s">
+        <v>682</v>
+      </c>
       <c r="M153" s="7"/>
       <c r="N153" s="7"/>
       <c r="O153" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O153" xr:uid="{4892E0D7-B48B-4F9C-BCDE-FF1B7E06E61D}"/>
+  <conditionalFormatting sqref="C2:E153">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2AF78BD6-C24F-4662-A21D-CFDBCF7BD100}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L153" xr:uid="{780CA5DA-AA5E-4D2F-A0C9-DA681E5C8085}">
       <formula1>"OK as suggested,Keep English,Translate,English name + Spanish noun"</formula1>
@@ -7989,6 +8647,23 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{2AF78BD6-C24F-4662-A21D-CFDBCF7BD100}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>C2:E153</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -8005,7 +8680,7 @@
     <col min="6" max="6" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>587</v>
       </c>
@@ -8038,7 +8713,9 @@
       <c r="D2" s="4" t="s">
         <v>593</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F2" s="8"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -8054,7 +8731,9 @@
       <c r="D3" s="4" t="s">
         <v>597</v>
       </c>
-      <c r="E3" s="8"/>
+      <c r="E3" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F3" s="8"/>
     </row>
     <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8070,7 +8749,9 @@
       <c r="D4" s="4" t="s">
         <v>601</v>
       </c>
-      <c r="E4" s="8"/>
+      <c r="E4" s="8" t="s">
+        <v>740</v>
+      </c>
       <c r="F4" s="8"/>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8086,7 +8767,9 @@
       <c r="D5" s="4" t="s">
         <v>605</v>
       </c>
-      <c r="E5" s="8"/>
+      <c r="E5" s="8" t="s">
+        <v>742</v>
+      </c>
       <c r="F5" s="8"/>
     </row>
     <row r="6" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8102,10 +8785,12 @@
       <c r="D6" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="E6" s="8"/>
+      <c r="E6" s="8" t="s">
+        <v>743</v>
+      </c>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>610</v>
       </c>
@@ -8118,8 +8803,12 @@
       <c r="D7" s="4" t="s">
         <v>613</v>
       </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+      <c r="E7" s="8" t="s">
+        <v>741</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>744</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -8134,7 +8823,9 @@
       <c r="D8" s="4" t="s">
         <v>617</v>
       </c>
-      <c r="E8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8150,8 +8841,12 @@
       <c r="D9" s="4" t="s">
         <v>621</v>
       </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
+      <c r="E9" s="8" t="s">
+        <v>739</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>745</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
@@ -8166,7 +8861,9 @@
       <c r="D10" s="4" t="s">
         <v>625</v>
       </c>
-      <c r="E10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -8182,7 +8879,9 @@
       <c r="D11" s="4" t="s">
         <v>629</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8196,7 +8895,9 @@
         <v>632</v>
       </c>
       <c r="D12" s="4"/>
-      <c r="E12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -8212,7 +8913,9 @@
       <c r="D13" s="4" t="s">
         <v>636</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -8228,7 +8931,9 @@
       <c r="D14" s="4" t="s">
         <v>640</v>
       </c>
-      <c r="E14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -8244,7 +8949,9 @@
       <c r="D15" s="4" t="s">
         <v>644</v>
       </c>
-      <c r="E15" s="8"/>
+      <c r="E15" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="38.25" x14ac:dyDescent="0.2">
@@ -8260,7 +8967,9 @@
       <c r="D16" s="4" t="s">
         <v>648</v>
       </c>
-      <c r="E16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8276,7 +8985,9 @@
       <c r="D17" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="E17" s="8"/>
+      <c r="E17" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8292,7 +9003,9 @@
       <c r="D18" s="4" t="s">
         <v>656</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
@@ -8306,7 +9019,9 @@
         <v>659</v>
       </c>
       <c r="D19" s="4"/>
-      <c r="E19" s="8"/>
+      <c r="E19" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="38.25" x14ac:dyDescent="0.2">
@@ -8322,7 +9037,9 @@
       <c r="D20" s="4" t="s">
         <v>663</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>739</v>
+      </c>
       <c r="F20" s="8"/>
     </row>
   </sheetData>

</xml_diff>